<commit_message>
update them cot So luong scan
</commit_message>
<xml_diff>
--- a/templates/mau_bao_cao_hop_dong_ctv.xlsx
+++ b/templates/mau_bao_cao_hop_dong_ctv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\programme\git_repository\bmk\bmk-ctv-service\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D3B56FF-13A6-485D-8C18-153DFCEABF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431756BD-0899-4F29-B172-4C3EC45BC466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Báo cáo HĐ" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="12">
   <si>
     <t>STT</t>
   </si>
@@ -52,7 +52,10 @@
     <t>Hợp đồng 5</t>
   </si>
   <si>
-    <t>Số lượng</t>
+    <t>Số lượng excel</t>
+  </si>
+  <si>
+    <t>Số lượng Scan</t>
   </si>
 </sst>
 </file>
@@ -196,10 +199,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -208,7 +208,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -546,99 +549,102 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:N29"/>
+  <dimension ref="A2:O29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.7265625" customWidth="1"/>
     <col min="2" max="2" width="15.1796875" style="3" customWidth="1"/>
-    <col min="3" max="4" width="22.7265625" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="14.90625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="13.81640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="15.1796875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="14.1796875" style="3" customWidth="1"/>
-    <col min="10" max="10" width="15.1796875" style="3" customWidth="1"/>
-    <col min="11" max="11" width="15.54296875" style="3" customWidth="1"/>
-    <col min="12" max="12" width="14.90625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="15.54296875" style="3" customWidth="1"/>
-    <col min="14" max="14" width="14.90625" style="3" customWidth="1"/>
-    <col min="15" max="15" width="16.1796875" customWidth="1"/>
-    <col min="16" max="16" width="27.1796875" customWidth="1"/>
+    <col min="3" max="5" width="22.7265625" customWidth="1"/>
+    <col min="6" max="6" width="15.26953125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="14.90625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="13.81640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="15.1796875" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14.1796875" style="3" customWidth="1"/>
+    <col min="11" max="11" width="15.1796875" style="3" customWidth="1"/>
+    <col min="12" max="12" width="15.54296875" style="3" customWidth="1"/>
+    <col min="13" max="13" width="14.90625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="15.54296875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="14.90625" style="3" customWidth="1"/>
+    <col min="16" max="16" width="16.1796875" customWidth="1"/>
+    <col min="17" max="17" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="9"/>
+      <c r="H2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="9"/>
+      <c r="J2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="9"/>
+      <c r="L2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="6"/>
-      <c r="M2" s="9" t="s">
+      <c r="M2" s="9"/>
+      <c r="N2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="9"/>
-    </row>
-    <row r="3" spans="1:14" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="1" t="s">
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" spans="1:15" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="2"/>
-      <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -648,10 +654,10 @@
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O4" s="4"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B5" s="2"/>
-      <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -661,10 +667,10 @@
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O5" s="4"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B6" s="2"/>
-      <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -674,10 +680,10 @@
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O6" s="4"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B7" s="2"/>
-      <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -687,10 +693,10 @@
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O7" s="4"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B8" s="2"/>
-      <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -700,10 +706,10 @@
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O8" s="4"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B9" s="2"/>
-      <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -713,10 +719,10 @@
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O9" s="4"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B10" s="2"/>
-      <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -726,10 +732,10 @@
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O10" s="4"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B11" s="2"/>
-      <c r="E11" s="4"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -739,10 +745,10 @@
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O11" s="4"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B12" s="2"/>
-      <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -752,10 +758,10 @@
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="O12" s="4"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B13" s="2"/>
-      <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -765,9 +771,9 @@
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="E14" s="4"/>
+      <c r="O13" s="4"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -777,9 +783,9 @@
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="E15" s="4"/>
+      <c r="O14" s="4"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -789,9 +795,9 @@
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="E16" s="4"/>
+      <c r="O15" s="4"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -801,9 +807,9 @@
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
       <c r="N16" s="4"/>
-    </row>
-    <row r="17" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E17" s="4"/>
+      <c r="O16" s="4"/>
+    </row>
+    <row r="17" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -813,9 +819,9 @@
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
-    </row>
-    <row r="18" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E18" s="4"/>
+      <c r="O17" s="4"/>
+    </row>
+    <row r="18" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -825,9 +831,9 @@
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
-    </row>
-    <row r="19" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E19" s="4"/>
+      <c r="O18" s="4"/>
+    </row>
+    <row r="19" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -837,9 +843,9 @@
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
       <c r="N19" s="4"/>
-    </row>
-    <row r="20" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E20" s="4"/>
+      <c r="O19" s="4"/>
+    </row>
+    <row r="20" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -849,9 +855,9 @@
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
       <c r="N20" s="4"/>
-    </row>
-    <row r="21" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E21" s="4"/>
+      <c r="O20" s="4"/>
+    </row>
+    <row r="21" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -861,9 +867,9 @@
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
-    </row>
-    <row r="22" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E22" s="4"/>
+      <c r="O21" s="4"/>
+    </row>
+    <row r="22" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -873,9 +879,9 @@
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
-    </row>
-    <row r="23" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E23" s="4"/>
+      <c r="O22" s="4"/>
+    </row>
+    <row r="23" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -885,9 +891,9 @@
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
       <c r="N23" s="4"/>
-    </row>
-    <row r="24" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E24" s="4"/>
+      <c r="O23" s="4"/>
+    </row>
+    <row r="24" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
@@ -897,9 +903,9 @@
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
       <c r="N24" s="4"/>
-    </row>
-    <row r="25" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E25" s="4"/>
+      <c r="O24" s="4"/>
+    </row>
+    <row r="25" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -909,9 +915,9 @@
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
       <c r="N25" s="4"/>
-    </row>
-    <row r="26" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E26" s="4"/>
+      <c r="O25" s="4"/>
+    </row>
+    <row r="26" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
@@ -921,9 +927,9 @@
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
       <c r="N26" s="4"/>
-    </row>
-    <row r="27" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E27" s="4"/>
+      <c r="O26" s="4"/>
+    </row>
+    <row r="27" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
@@ -933,9 +939,9 @@
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
       <c r="N27" s="4"/>
-    </row>
-    <row r="28" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E28" s="4"/>
+      <c r="O27" s="4"/>
+    </row>
+    <row r="28" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -945,9 +951,9 @@
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
-    </row>
-    <row r="29" spans="5:14" x14ac:dyDescent="0.35">
-      <c r="E29" s="4"/>
+      <c r="O28" s="4"/>
+    </row>
+    <row r="29" spans="6:15" x14ac:dyDescent="0.35">
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -957,18 +963,20 @@
       <c r="L29" s="4"/>
       <c r="M29" s="4"/>
       <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="M2:N2"/>
+  <mergeCells count="10">
+    <mergeCell ref="N2:O2"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="L2:M2"/>
     <mergeCell ref="D2:D3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="K2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>